<commit_message>
Update DBMS content visuals and upload links
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Python/Unit 1 - Introduction to Programming/Unit 1 - Introduction to Programming - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Python/Unit 1 - Introduction to Programming/Unit 1 - Introduction to Programming - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 1" sheetId="1" r:id="Rd023f3486ef24f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 1" sheetId="1" r:id="R04432e9a816e43d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -460,20 +460,21 @@
         <x:v>Python - MCQ - 1.1.1</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>A student writes steps for a robot to make toast: (1) put the bread in the toaster, (2) press the lever, (3) spread butter on the toast. The robot burns itself trying to butter bread that is still inside the running toaster.
-Which quality of good instructions is missing?</x:v>
+        <x:v>A college uses a computer to prepare admission receipts. The draft instruction says:
+&gt; Work out the fee after tax and scholarship, then make a good receipt.
+The computer needs exact steps. Which instruction can it follow correctly every time?</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Good instructions must be unambiguous, ordered, and complete. Here a required step — taking the toast out before buttering it — was never written, so the steps are not complete. A literal machine will not add a step you left out.</x:v>
+        <x:v>It supplies clear inputs, a clear calculation, ordered steps, and a clear output rather than asking the computer to use judgment.</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E2" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G2" t="str">
         <x:v>analyze</x:v>
@@ -488,23 +489,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>what-is-programming</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L2"/>
       <x:c r="M2" t="str">
-        <x:v>Incomplete instructions</x:v>
+        <x:v>Prepare each receipt as quickly as possible and avoid mistakes</x:v>
       </x:c>
       <x:c r="N2" t="str">
-        <x:v>Ambiguous instructions</x:v>
+        <x:v>Read the student's details, calculate a fair amount, and print it neatly</x:v>
       </x:c>
       <x:c r="O2" t="str">
-        <x:v>Excessively detailed instructions</x:v>
+        <x:v>Read the base fee and scholarship, calculate `base fee + 18% tax - scholarship`, then print the name and amount</x:v>
       </x:c>
       <x:c r="P2" t="str">
-        <x:v>Instructions in the wrong language</x:v>
+        <x:v>Ask an experienced clerk to decide how every receipt should be calculated</x:v>
       </x:c>
       <x:c r="Q2" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="18" customHeight="1">
@@ -512,23 +513,22 @@
         <x:v>Python - MCQ - 1.1.2</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>A fitness band reads your steps from a sensor, works out how many calories you burned, and shows that number on its screen.
-In the IPO model, what is "working out the calories"?</x:v>
+        <x:v>A clerk can manually prepare one accurate receipt in two minutes. The college needs 5,000 receipts that follow the same rules. Which option best shows how programming can help?</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>IPO stands for Input, Processing, Output. Reading the sensor is input and showing the number is output. Working out the calories is a calculation done on the input, which is the processing stage.</x:v>
+        <x:v>Programming captures the rules once as instructions the computer can run so the machine can follow the same rules correctly many times.</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E3" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H3" t="str">
         <x:v>python - Set 1</x:v>
@@ -540,23 +540,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>inputs-processing-outputs</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L3"/>
       <x:c r="M3" t="str">
-        <x:v>Input stage</x:v>
+        <x:v>Write the receipt rules once as clear steps and let the computer use them for every student</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>Processing stage</x:v>
+        <x:v>Ask the clerk to memorise the rules so each receipt becomes slightly faster</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>Output stage</x:v>
+        <x:v>Scan one completed receipt 5,000 times</x:v>
       </x:c>
       <x:c r="P3" t="str">
-        <x:v>Long-term storage stage</x:v>
+        <x:v>Buy a faster printer without describing how each amount should be calculated</x:v>
       </x:c>
       <x:c r="Q3" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -564,20 +564,19 @@
         <x:v>Python - MCQ - 1.1.3</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>While planning a college fest, an organiser notices that printing certificates, printing fee receipts, and printing ID cards are all the same "one record per person" job — so one solution can be reused for all three.
-Which pillar of computational thinking is this?</x:v>
+        <x:v>Four interns describe their work on a shopping application. Which intern is programming, not just using the app?</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Noticing that different tasks share the same underlying shape, so one solution can be reused, is pattern recognition. Decomposition is splitting a big job into smaller ones, and abstraction is dropping details that do not matter.</x:v>
+        <x:v>Writing the instructions behind the button is writing software; the other interns are using features that already exist.</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E4" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G4" t="str">
         <x:v>understand</x:v>
@@ -592,23 +591,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>computational-thinking</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L4"/>
       <x:c r="M4" t="str">
-        <x:v>Splitting the task into smaller components</x:v>
+        <x:v>Meera taps “Add to Cart” to buy a notebook</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>Removing nonessential details</x:v>
+        <x:v>Faisal changes his delivery address through the settings screen</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>Recognising a repeated task pattern</x:v>
+        <x:v>Kavya uses the Download button to save her order history</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>Correcting an existing program</x:v>
+        <x:v>Arjun writes the steps that check an item, update the cart, and show the new quantity</x:v>
       </x:c>
       <x:c r="Q4" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -616,20 +615,19 @@
         <x:v>Python - MCQ - 1.1.4</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>An algorithm for cooking includes the step "season the dish somehow". A classmate says this cannot be a proper algorithm step.
-Which property does that step break?</x:v>
+        <x:v>An automated pharmacy cabinet must dispense medicine only for a valid prescription. Which sequence is complete and in the correct order?</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Definiteness means every step has exactly one meaning. "Somehow" can be read in many ways, so two people could do it differently — that breaks definiteness. It is not about the step running forever (finiteness) or lacking data (input).</x:v>
+        <x:v>It gathers and verifies the required information before selecting and dispensing the prescribed medicine.</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E5" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G5" t="str">
         <x:v>analyze</x:v>
@@ -644,20 +642,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>algorithms</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L5"/>
       <x:c r="M5" t="str">
-        <x:v>Finiteness</x:v>
+        <x:v>Dispense medicine → read prescription → confirm patient</x:v>
       </x:c>
       <x:c r="N5" t="str">
-        <x:v>Definiteness</x:v>
+        <x:v>Read patient ID → read prescription → verify patient and prescription → select prescribed medicine → dispense it</x:v>
       </x:c>
       <x:c r="O5" t="str">
-        <x:v>Output</x:v>
+        <x:v>Select any available medicine → check whether the patient wants it → dispense</x:v>
       </x:c>
       <x:c r="P5" t="str">
-        <x:v>Effectiveness</x:v>
+        <x:v>Read patient ID → dispense medicine → verify the prescription later</x:v>
       </x:c>
       <x:c r="Q5" t="n">
         <x:v>2</x:v>
@@ -668,28 +666,22 @@
         <x:v>Python - MCQ - 1.1.5</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>A beginner runs this program and says "only two lines appear, so something must be broken":
-```python
-print("Start")
-total = 40 + 2
-print("Total is", total)
-```
-How many lines appear, and is anything broken?</x:v>
+        <x:v>A taxi application receives the travelled distance and price per kilometre, calculates the fare, and displays the amount due. Which IPO description matches the system?</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>`print("Start")` shows one line, and `print("Total is", total)` shows `Total is 42`. The middle line only stores a value, which is processing, not output, so it shows nothing. Two lines is exactly right — nothing is broken.</x:v>
+        <x:v>Distance and rate enter the program, multiplication transforms them, and the fare is the result returned to the user.</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E6" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H6" t="str">
         <x:v>python - Set 1</x:v>
@@ -701,23 +693,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>setting-up-python-first-program</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L6"/>
       <x:c r="M6" t="str">
-        <x:v>Two lines</x:v>
+        <x:v>Input: calculated fare; Processing: display it; Output: distance and rate</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>Three lines</x:v>
+        <x:v>Input: multiplication; Processing: fare due; Output: distance</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>One line</x:v>
+        <x:v>Input: distance and rate; Processing: multiply them; Output: fare due</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>No lines</x:v>
+        <x:v>Input: passenger name only; Processing: save the name; Output: distance</x:v>
       </x:c>
       <x:c r="Q6" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -725,23 +717,22 @@
         <x:v>Python - MCQ - 1.1.6</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>In a flowchart, one shape marks a yes/no question where the path splits into two branches.
-Which shape is it?</x:v>
+        <x:v>A team receives the large task “build a hospital appointment system.” Which option correctly breaks the system into smaller parts?</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>A diamond marks a decision — a yes/no question that splits the path. An oval starts or ends the chart, a rectangle is a plain process step, and a parallelogram is for input or output.</x:v>
+        <x:v>Decomposition makes the large system manageable by identifying clear smaller problems.</x:v>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E7" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>remember</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H7" t="str">
         <x:v>python - Set 1</x:v>
@@ -753,23 +744,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>flowcharts</x:v>
+        <x:v>computational-thinking</x:v>
       </x:c>
       <x:c r="L7"/>
       <x:c r="M7" t="str">
-        <x:v>Oval</x:v>
+        <x:v>Choose the colour of every screen before identifying what the system must do</x:v>
       </x:c>
       <x:c r="N7" t="str">
-        <x:v>Rectangle</x:v>
+        <x:v>Treat the entire system as one task so no component is considered separately</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>Diamond</x:v>
+        <x:v>Write the final program immediately and discover the required features later</x:v>
       </x:c>
       <x:c r="P7" t="str">
-        <x:v>Parallelogram</x:v>
+        <x:v>Split the system into registration, doctor availability, booking, cancellation, and reminders</x:v>
       </x:c>
       <x:c r="Q7" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -777,23 +768,15 @@
         <x:v>Python - MCQ - 1.1.7</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Read this pseudocode:
-```
-READ mark1, mark2, mark3
-SET average = (mark1 + mark2 + mark3) / 3
-IF average &gt;= 40 THEN
-    PRINT "Pass"
-ELSE
-    PRINT "Fail"
-END IF
-```
-For marks 30, 35, and 30, what does it print?</x:v>
+        <x:v>A route algorithm contains this step:
+&gt; Arrange all deliveries properly before starting.
+Two drivers interpret “properly” differently. Which property of a good algorithm is missing?</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Add the marks: 30 + 35 + 30 = 95. Divide by 3 to get about 31.7. Since 31.7 is below 40, the `IF` is false and the `ELSE` runs, printing `Fail`. Pseudocode can be traced by hand exactly like this.</x:v>
+        <x:v>“Properly” allows different interpretations, so the step is not definite.</x:v>
       </x:c>
       <x:c r="D8" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>published</x:v>
@@ -802,7 +785,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>apply</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H8" t="str">
         <x:v>python - Set 1</x:v>
@@ -814,23 +797,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>pseudocode</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L8"/>
       <x:c r="M8" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="N8" t="str">
-        <x:v>Pass</x:v>
+        <x:v>Definiteness</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>No message</x:v>
+        <x:v>Output</x:v>
       </x:c>
       <x:c r="P8" t="str">
-        <x:v>Pass and Fail</x:v>
+        <x:v>Finiteness</x:v>
       </x:c>
       <x:c r="Q8" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -838,14 +821,13 @@
         <x:v>Python - MCQ - 1.1.8</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>A beginner is surprised that Python code to greet three friends reads almost like an English sentence, while the same task in many older languages first needs type declarations, semicolons, and curly braces.
-What makes Python read so cleanly?</x:v>
+        <x:v>A refund workflow contains several approval decisions, a path back for missing documents, and an audience of non-technical store managers. Which tool is best for the meeting?</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Python's designers chose English-like keywords, very little boilerplate, and indentation that is part of the language itself. This keeps the code and the idea behind it looking almost the same, instead of burying the idea under punctuation.</x:v>
+        <x:v>A flowchart makes pathes, loops, and return paths visible to technical and non-technical readers.</x:v>
       </x:c>
       <x:c r="D9" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E9" t="str">
         <x:v>published</x:v>
@@ -854,7 +836,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H9" t="str">
         <x:v>python - Set 1</x:v>
@@ -866,23 +848,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>why-python</x:v>
+        <x:v>flowcharts</x:v>
       </x:c>
       <x:c r="L9"/>
       <x:c r="M9" t="str">
-        <x:v>Removing every keyword</x:v>
+        <x:v>Executable Python with no diagram</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>Compiling before execution</x:v>
+        <x:v>A flowchart with decisions, labelled paths, and a return arrow</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>Restricting every program to short learning scripts</x:v>
+        <x:v>A long paragraph with every branch embedded in sentences</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>Readable keywords and meaningful indentation</x:v>
+        <x:v>A screenshot of the final refund screen</x:v>
       </x:c>
       <x:c r="Q9" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -890,14 +872,13 @@
         <x:v>Python - MCQ - 1.1.9</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>A program asks for a number using `input()`, and the user types 25. A student expects Python to store the number 25 so it can do maths with it right away.
-What does Python actually store, and why does it matter?</x:v>
+        <x:v>A teaching team wants beginners to focus on problem-solving rather than a lot of complex syntax, while still learning a language used in automation, data, web systems, and AI. Why is Python a good choice?</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>`input()` always hands back plain text, so Python stores the text `"25"`, not the number 25. Before doing any maths you must convert it to a number first. This is a detail the next unit builds on directly.</x:v>
+        <x:v>Python combines simple syntax and readability with many useful libraries and real-world uses.</x:v>
       </x:c>
       <x:c r="D10" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E10" t="str">
         <x:v>published</x:v>
@@ -918,23 +899,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>setting-up-python-first-program</x:v>
+        <x:v>python-overview</x:v>
       </x:c>
       <x:c r="L10"/>
       <x:c r="M10" t="str">
-        <x:v>The number 25</x:v>
+        <x:v>Its syntax is easy to read, and it is useful for many real projects</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>No stored value</x:v>
+        <x:v>Python guarantees that beginners will never encounter errors</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>The number 25.0</x:v>
+        <x:v>Python is the fastest possible language for every kind of software</x:v>
       </x:c>
       <x:c r="P10" t="str">
-        <x:v>The text "25"</x:v>
+        <x:v>Python requires no interpreter or runtime</x:v>
       </x:c>
       <x:c r="Q10" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -942,23 +923,22 @@
         <x:v>Python - MCQ - 1.1.10</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>A pass/fail rule says "an average of 40 or more passes". A careful student wants the one test case most likely to catch a mistake where someone wrote `&gt;` instead of `&gt;=`.
-Which set of marks should they test?</x:v>
+        <x:v>A student wants to calculate `1234 × 5678` once and does not need to keep the work. Which Python workspace is best?</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>The `&gt;` vs `&gt;=` mistake only shows up right at the pass mark. Marks of 40, 40, 40 give an average of exactly 40, which must pass under "40 or more" but would wrongly fail if `&gt;` were used. Clearly-passing or clearly-failing marks cannot reveal that mistake.</x:v>
+        <x:v>The REPL is intended for quick tests that do not need to be saved and calculations.</x:v>
       </x:c>
       <x:c r="D11" t="n">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E11" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>hard</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H11" t="str">
         <x:v>python - Set 1</x:v>
@@ -970,23 +950,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>problem-solving-approach</x:v>
+        <x:v>python-environment</x:v>
       </x:c>
       <x:c r="L11"/>
       <x:c r="M11" t="str">
-        <x:v>90, 85, 95</x:v>
+        <x:v>The REPL, because it gives an immediate answer and the session need not be saved</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>40, 40, 40</x:v>
+        <x:v>A saved package containing several files</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>10, 5, 0</x:v>
+        <x:v>A permanent script that must be reopened next semester</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>1000, 100, 100</x:v>
+        <x:v>A flowchart, because flowcharts execute calculations</x:v>
       </x:c>
       <x:c r="Q11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -994,14 +974,13 @@
         <x:v>Python - MCQ - 1.2.1</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Consider two actions: tapping "Add to Cart" on a shopping app, and writing the logic that runs the moment that button is tapped.
-Which one is writing software?</x:v>
+        <x:v>A backup application begins automatically every night at 2:00 AM. No user clicks a button. In the IPO model, what is the input?</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Using software means following choices someone already built, like tapping a button. Writing software means deciding what those steps should be — writing the logic behind the button. So writing the logic is programming.</x:v>
+        <x:v>Input can be a scheduled trigger; it does not require a person typing or clicking.</x:v>
       </x:c>
       <x:c r="D12" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E12" t="str">
         <x:v>published</x:v>
@@ -1010,7 +989,7 @@
         <x:v>easy</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H12" t="str">
         <x:v>python - Set 2</x:v>
@@ -1022,20 +1001,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>what-is-programming</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L12"/>
       <x:c r="M12" t="str">
-        <x:v>Using the existing Add to Cart button</x:v>
+        <x:v>The completion message shown after the backup</x:v>
       </x:c>
       <x:c r="N12" t="str">
-        <x:v>Both activities</x:v>
+        <x:v>The CPU performing the copy</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>Neither activity</x:v>
+        <x:v>The copied files stored at the destination</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>Writing the button's behaviour</x:v>
+        <x:v>The scheduled 2:00 AM trigger</x:v>
       </x:c>
       <x:c r="Q12" t="n">
         <x:v>4</x:v>
@@ -1046,14 +1025,13 @@
         <x:v>Python - MCQ - 1.2.2</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>A helper follows instructions exactly and never fills in a step you leave out. You tell it: spread the butter, put the second slice on top, serve — but you forget the step "take out two slices of bread first".
-What does this literal helper do?</x:v>
+        <x:v>A parcel service uses a correct formula to calculate delivery charges from weight. One scale sends `650` for a 650-gram parcel, while a faulty scale sends `6500`. The software charges ten times too much. What should the parcel service fix?</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>A computer, like the literal helper, follows instructions exactly as written and never adds a missing step. With no bread taken out, it tries to spread butter on nothing. It does not guess your intention or fix the gap for you.</x:v>
+        <x:v>Correct processing cannot rescue a faulty weight. Checking the input addresses the garbage-in, garbage-out problem.</x:v>
       </x:c>
       <x:c r="D13" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E13" t="str">
         <x:v>published</x:v>
@@ -1062,7 +1040,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H13" t="str">
         <x:v>python - Set 2</x:v>
@@ -1074,23 +1052,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K13" t="str">
-        <x:v>what-is-programming</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L13"/>
       <x:c r="M13" t="str">
-        <x:v>It retrieves bread by itself</x:v>
+        <x:v>Check that the weight is reasonable before using the formula</x:v>
       </x:c>
       <x:c r="N13" t="str">
-        <x:v>It requests the missing step</x:v>
+        <x:v>Replace the output screen because it displayed the charge accurately</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>It rearranges the steps automatically</x:v>
+        <x:v>Make the CPU repeat the same calculation twice</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>It tries to butter without bread</x:v>
+        <x:v>Move the charge calculation from processing into output</x:v>
       </x:c>
       <x:c r="Q13" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1098,23 +1076,22 @@
         <x:v>Python - MCQ - 1.2.3</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>An exam portal is given a student's mark as the word "ninety" instead of the number 90. The processing logic is flawless, yet the final result is wrong.
-Which idea does this show?</x:v>
+        <x:v>A note-taking program keeps a new paragraph available while the program is open, but the paragraph disappears after a power failure because the user never saved it. Why was the paragraph lost?</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>"Garbage in, garbage out" means that even perfect processing cannot rescue bad input — a wrong or badly-shaped input leads to a wrong output. This is exactly why careful programs check their input before trusting it.</x:v>
+        <x:v>RAM holds active data temporarily and loses it when power ends; only deliberately saved data survives in storage.</x:v>
       </x:c>
       <x:c r="D14" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E14" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H14" t="str">
         <x:v>python - Set 2</x:v>
@@ -1126,23 +1103,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K14" t="str">
-        <x:v>inputs-processing-outputs</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L14"/>
       <x:c r="M14" t="str">
-        <x:v>Bad input can spoil the result</x:v>
+        <x:v>The paragraph was stored permanently by the CPU</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>The steps may never finish</x:v>
+        <x:v>The keyboard deleted the paragraph when power stopped</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>Unimportant details were removed</x:v>
+        <x:v>The paragraph existed only in RAM, and it was never written to long-term storage</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>Output should be designed first</x:v>
+        <x:v>The screen was responsible for remembering the paragraph</x:v>
       </x:c>
       <x:c r="Q14" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1150,23 +1127,22 @@
         <x:v>Python - MCQ - 1.2.4</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>While a program runs, it holds the PIN you just typed, but loses it the moment the program closes.
-Which part of the computer holds data that disappears like this?</x:v>
+        <x:v>An ATM receives a PIN, checks it, shows an approval message, and records the completed transaction for future visits. Which mapping is correct?</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>RAM is short-term memory: it holds the data a program is actively using but is cleared when the program closes. Storage keeps files even with the power off, and the CPU does the calculations rather than holding working data.</x:v>
+        <x:v>The keypad is an input device, the CPU processes, the screen outputs, and storage preserves the transaction.</x:v>
       </x:c>
       <x:c r="D15" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E15" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H15" t="str">
         <x:v>python - Set 2</x:v>
@@ -1178,20 +1154,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K15" t="str">
-        <x:v>inputs-processing-outputs</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L15"/>
       <x:c r="M15" t="str">
-        <x:v>CPU — hardware that performs calculations</x:v>
+        <x:v>Screen checks the PIN; CPU stores the permanent record; keypad shows approval</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>RAM — temporary working memory</x:v>
+        <x:v>Keypad supplies input; CPU performs the check; screen supplies output; storage keeps the lasting record</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>Storage — long-term memory</x:v>
+        <x:v>Storage reads the PIN; RAM dispenses cash; keypad performs the comparison</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>Keypad — input hardware</x:v>
+        <x:v>CPU supplies the PIN; screen processes it; storage displays approval</x:v>
       </x:c>
       <x:c r="Q15" t="n">
         <x:v>2</x:v>
@@ -1202,23 +1178,22 @@
         <x:v>Python - MCQ - 1.2.5</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>Nobody writes a whole banking app in one go. It is split into login, balance, transfer, and statements, and each of those is split further until every piece is small enough to build.
-Which pillar of computational thinking is this?</x:v>
+        <x:v>A college separately prints fee receipts, ID cards, and course certificates. A developer notices that each task reads one student record, fills a template, and produces one personalised document. How should the developer use this repeated pattern?</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>Breaking a big, overwhelming problem into smaller, manageable sub-problems is decomposition. Abstraction is dropping unimportant detail, and pattern recognition is spotting repeated shapes of task.</x:v>
+        <x:v>The shared record-to-document pattern can be solved once and reused with different templates.</x:v>
       </x:c>
       <x:c r="D16" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E16" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H16" t="str">
         <x:v>python - Set 2</x:v>
@@ -1234,19 +1209,19 @@
       </x:c>
       <x:c r="L16"/>
       <x:c r="M16" t="str">
-        <x:v>Abstraction</x:v>
+        <x:v>Ignore the shared steps because the documents have different names</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>Pattern recognition</x:v>
+        <x:v>Create one reusable process and use the correct template for each document</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>Efficiency</x:v>
+        <x:v>Merge every document into one identical design</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>Decomposition</x:v>
+        <x:v>Ask students to create all three documents manually</x:v>
       </x:c>
       <x:c r="Q16" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1254,14 +1229,13 @@
         <x:v>Python - MCQ - 1.2.6</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>A friend claims the plain-English steps for finding the largest of three numbers and the Python version of it are two completely unrelated things.
-Which statement is correct?</x:v>
+        <x:v>A team is planning how to estimate the arrival time for a food order. Which set keeps the needed details and removes unneeded ones?</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>An algorithm is the language-independent plan written in plain steps. A program is that same plan written in one specific language. So the English steps are the algorithm, and the Python version is one program that implements it.</x:v>
+        <x:v>Those details directly affect arrival time; the other choices retain irrelevant personal or visual details.</x:v>
       </x:c>
       <x:c r="D17" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E17" t="str">
         <x:v>published</x:v>
@@ -1270,7 +1244,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H17" t="str">
         <x:v>python - Set 2</x:v>
@@ -1282,23 +1256,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>algorithms</x:v>
+        <x:v>computational-thinking</x:v>
       </x:c>
       <x:c r="L17"/>
       <x:c r="M17" t="str">
-        <x:v>The two descriptions are unrelated</x:v>
+        <x:v>Distance, current traffic, preparation time, and rider availability</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>Only executable Python code qualifies as an algorithm</x:v>
+        <x:v>Customer's wallpaper, rider's shirt colour, and restaurant logo</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>One is the plan; the other implements it</x:v>
+        <x:v>Customer's favourite cuisine, phone model, and profile photo</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>Both must be written in Python</x:v>
+        <x:v>Every detail stored about the customer, restaurant, and rider</x:v>
       </x:c>
       <x:c r="Q17" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1306,20 +1280,19 @@
         <x:v>Python - MCQ - 1.2.7</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>A set of steps keeps repeating and has no way to ever stop.
-Why is this not a true algorithm?</x:v>
+        <x:v>A clinic scheduler keeps doctor name, patient name, and appointment date, but removes appointment duration to “simplify” the model. Later it assigns two patients to the same doctor at overlapping times. What is the best conclusion?</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>Every algorithm must be finite — guaranteed to stop after a limited number of steps. Steps that could run forever break finiteness, which is exactly why infinite loops are treated as bugs. The steps here may be perfectly clear, so definiteness is not the issue.</x:v>
+        <x:v>Duration is essential to checking overlap. Abstraction simplifies only by removing details that do not affect the solution.</x:v>
       </x:c>
       <x:c r="D18" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E18" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F18" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G18" t="str">
         <x:v>analyze</x:v>
@@ -1334,23 +1307,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>algorithms</x:v>
+        <x:v>computational-thinking</x:v>
       </x:c>
       <x:c r="L18"/>
       <x:c r="M18" t="str">
-        <x:v>Finiteness</x:v>
+        <x:v>The model needs more decorative patient information</x:v>
       </x:c>
       <x:c r="N18" t="str">
-        <x:v>Definiteness</x:v>
+        <x:v>The model removed the appointment duration, which is needed to find overlaps</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>Input</x:v>
+        <x:v>Decomposition should never be used with scheduling problems</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>No algorithm property</x:v>
+        <x:v>Pattern recognition caused the scheduler to forget the date</x:v>
       </x:c>
       <x:c r="Q18" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1358,23 +1331,22 @@
         <x:v>Python - MCQ - 1.2.8</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>After building a program, a developer tests it with unusual inputs like all zeros and a value sitting exactly on the boundary, then improves it based on what they find.
-Which stage of the four-stage problem-solving method is this?</x:v>
+        <x:v>A festival team handles workshop entry, meal coupons, and certificates separately. A new plan splits registration into services, notices that each service checks the same student ID, and removes clothing colour. Which statement is correct?</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>The four stages are Understand, Plan, Carry Out, and Look Back. Testing with tricky inputs and improving the result is the Look Back stage — the step many beginners skip, and the one that catches subtle bugs.</x:v>
+        <x:v>The plan splits the workflow, reuses a repeated ID check, and removes an irrelevant detail.</x:v>
       </x:c>
       <x:c r="D19" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E19" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>python - Set 2</x:v>
@@ -1386,23 +1358,23 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K19" t="str">
-        <x:v>problem-solving-approach</x:v>
+        <x:v>computational-thinking</x:v>
       </x:c>
       <x:c r="L19"/>
       <x:c r="M19" t="str">
-        <x:v>Understand</x:v>
+        <x:v>It uses abstraction only</x:v>
       </x:c>
       <x:c r="N19" t="str">
-        <x:v>Plan</x:v>
+        <x:v>It uses decomposition and ignores pattern recognition</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>Carry Out</x:v>
+        <x:v>It combines decomposition, pattern recognition, and abstraction</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>Look Back</x:v>
+        <x:v>It uses pattern recognition but keeps every irrelevant detail</x:v>
       </x:c>
       <x:c r="Q19" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1410,14 +1382,13 @@
         <x:v>Python - MCQ - 1.2.9</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>In a login flowchart, an arrow points from "wrong password" back up to "read password" so the user can try again.
-What does a backward arrow represent?</x:v>
+        <x:v>A scholarship team reviews scores in this order: `72, 88, 65, 90, 77`. Its paper trace records the “highest so far” after each score is considered. Which trace is correct?</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>A backward arrow sends the flow to an earlier step so it runs again — that is repetition, which is a loop. It is the same idea you later write as a repeating loop in code.</x:v>
+        <x:v>The stored maximum progresses from 72 to 88, stays 88 for 65, becomes 90, and stays 90 for 77.</x:v>
       </x:c>
       <x:c r="D20" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E20" t="str">
         <x:v>published</x:v>
@@ -1426,7 +1397,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H20" t="str">
         <x:v>python - Set 2</x:v>
@@ -1438,20 +1409,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K20" t="str">
-        <x:v>flowcharts</x:v>
+        <x:v>computational-thinking</x:v>
       </x:c>
       <x:c r="L20"/>
       <x:c r="M20" t="str">
-        <x:v>A loop</x:v>
+        <x:v>`72, 88, 88, 90, 90`</x:v>
       </x:c>
       <x:c r="N20" t="str">
-        <x:v>The program ending</x:v>
+        <x:v>`72, 88, 65, 90, 77`</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>An input operation</x:v>
+        <x:v>`90, 90, 90, 90, 90`</x:v>
       </x:c>
       <x:c r="P20" t="str">
-        <x:v>A failed decision</x:v>
+        <x:v>`72, 72, 72, 72, 72`</x:v>
       </x:c>
       <x:c r="Q20" t="n">
         <x:v>1</x:v>
@@ -1462,14 +1433,13 @@
         <x:v>Python - MCQ - 1.2.10</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>A student removes all the indentation from working Python code to "tidy it up", and the code stops running.
-Why did that happen?</x:v>
+        <x:v>A client asks a team to “make the student search fast,” but does not state how many records exist, what users search by, or what response time is acceptable. What should the team do first?</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>In Python, indentation is part of the language, not just decoration — it shows which lines belong together. Remove it and Python can no longer tell the structure, so the code breaks. Python uses indentation where other languages use braces.</x:v>
+        <x:v>The team must understand and clarify the problem before planning or implementation can be reliable.</x:v>
       </x:c>
       <x:c r="D21" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E21" t="str">
         <x:v>published</x:v>
@@ -1490,38 +1460,37 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K21" t="str">
-        <x:v>why-python</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L21"/>
       <x:c r="M21" t="str">
-        <x:v>Semicolons define Python blocks</x:v>
+        <x:v>Build the search screen and decide the rules afterward</x:v>
       </x:c>
       <x:c r="N21" t="str">
-        <x:v>Indentation defines Python blocks</x:v>
+        <x:v>Select Python because implementation always comes first</x:v>
       </x:c>
       <x:c r="O21" t="str">
-        <x:v>Indentation matters only in older languages</x:v>
+        <x:v>Test a finished solution against random values</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>The original code was already invalid</x:v>
+        <x:v>Ask the client to clarify the inputs, output, limits, and the meaning of “fast”</x:v>
       </x:c>
       <x:c r="Q21" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>Python - MCQ - 1.2.11</x:v>
+        <x:v>Python - MCQ - 1.3.1</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>A teammate asks why you sketched pseudocode on the whiteboard instead of writing real code.
-What is the best reason?</x:v>
+        <x:v>Two students understand a pass/fail requirement. One starts typing immediately. The other lists the inputs, average calculation, threshold decision, and displayed result before opening an editor. Which problem-solving stage is the second student using?</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>Pseudocode captures an algorithm's logic in plain words plus a few keywords, written for humans to reason about — not for a computer to run. It lets you think about what should happen without fighting a language's exact syntax.</x:v>
+        <x:v>Listing the planned steps after understanding the requirement is the planning stage.</x:v>
       </x:c>
       <x:c r="D22" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E22" t="str">
         <x:v>published</x:v>
@@ -1530,10 +1499,10 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H22" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I22" t="str">
         <x:v>python</x:v>
@@ -1542,20 +1511,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K22" t="str">
-        <x:v>pseudocode</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L22"/>
       <x:c r="M22" t="str">
-        <x:v>Running logic faster than Python</x:v>
+        <x:v>Look back</x:v>
       </x:c>
       <x:c r="N22" t="str">
-        <x:v>Giving instructions directly to the computer</x:v>
+        <x:v>Carry out</x:v>
       </x:c>
       <x:c r="O22" t="str">
-        <x:v>Planning logic without exact syntax</x:v>
+        <x:v>Plan</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>Replacing all later implementation</x:v>
+        <x:v>Installation</x:v>
       </x:c>
       <x:c r="Q22" t="n">
         <x:v>3</x:v>
@@ -1563,29 +1532,28 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
-        <x:v>Python - MCQ - 1.2.12</x:v>
+        <x:v>Python - MCQ - 1.3.2</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>Abstraction means keeping the details that matter and dropping the rest. At a registration desk you keep the name and the ticket number, and ignore the colour of each student's shirt.
-What happens if you also abstract away the ticket number?</x:v>
+        <x:v>A scholarship is awarded when the average is **75 or more**. The solution works for 74 and 90. Which test best checks whether the rule includes the exact boundary?</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>Abstraction removes irrelevant detail, never important detail. The ticket number is essential to registration, so dropping it is dropping something that matters — and the solution quietly breaks. Shirt colour was safe to drop; the ticket number was not.</x:v>
+        <x:v>Testing exactly 75 distinguishes an rule that includes 75 from an wrong rule that starts above 75.</x:v>
       </x:c>
       <x:c r="D23" t="n">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E23" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F23" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G23" t="str">
         <x:v>analyze</x:v>
       </x:c>
       <x:c r="H23" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I23" t="str">
         <x:v>python</x:v>
@@ -1594,43 +1562,37 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K23" t="str">
-        <x:v>computational-thinking</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L23"/>
       <x:c r="M23" t="str">
-        <x:v>Nothing changes</x:v>
+        <x:v>Average `0`</x:v>
       </x:c>
       <x:c r="N23" t="str">
-        <x:v>The solution loses essential information</x:v>
+        <x:v>Average `1000`</x:v>
       </x:c>
       <x:c r="O23" t="str">
-        <x:v>The desk uses less data</x:v>
+        <x:v>Average `76`</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>The task becomes decomposition</x:v>
+        <x:v>Average `75`</x:v>
       </x:c>
       <x:c r="Q23" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
-        <x:v>Python - MCQ - 1.2.13</x:v>
+        <x:v>Python - MCQ - 1.3.3</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>Look at this program:
-```python
-print("Welcome!")
-score = 10 + 5
-print("Your score is", score)
-```
-Which line puts nothing on the screen, and why?</x:v>
+        <x:v>A booking plan should accept requests from 1 through 6 tickets. Which small test set checks a normal value, both limits, and values just outside the limits?</x:v>
       </x:c>
       <x:c r="C24" t="str">
-        <x:v>The first line prints `Welcome!` and the third prints `Your score is 15`. The middle line works out 15 and stores it in `score`, but storing a value is processing, not output — only `print` puts something on screen. So the middle line shows nothing.</x:v>
+        <x:v>It covers a typical valid value, both valid endpoints, and the closest invalid values below and above the range.</x:v>
       </x:c>
       <x:c r="D24" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E24" t="str">
         <x:v>published</x:v>
@@ -1639,10 +1601,10 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H24" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I24" t="str">
         <x:v>python</x:v>
@@ -1651,50 +1613,49 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K24" t="str">
-        <x:v>setting-up-python-first-program</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L24"/>
       <x:c r="M24" t="str">
-        <x:v>The first line</x:v>
+        <x:v>`2, 3, 4, 5, 6`</x:v>
       </x:c>
       <x:c r="N24" t="str">
-        <x:v>The third line</x:v>
+        <x:v>`0, 1, 3, 6, 7`</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>The middle line</x:v>
+        <x:v>`1, 1, 1, 1, 1`</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>All three lines</x:v>
+        <x:v>`-100, 100, 1000, 10000`</x:v>
       </x:c>
       <x:c r="Q24" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>Python - MCQ - 1.2.14</x:v>
+        <x:v>Python - MCQ - 1.3.4</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>To find "Ravi" among 10,000 contacts, you could check every name from the top, or jump straight to the R names and scan only those. Both always give the right answer.
-What is the main difference between them?</x:v>
+        <x:v>The task says, “Read all student records and display the best student.” The records contain marks, attendance, project score, and sports points. A developer chooses the highest marks without consulting anyone. What should the developer have done first?</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>Both approaches are correct, definite, and finite — they always find Ravi. The difference is efficiency: how quickly they finish. Jumping to the R names checks far fewer names, so it is much faster on a big list.</x:v>
+        <x:v>“Best” is ambiguous because several several measures are possible; the selection rule must be clarified during understanding.</x:v>
       </x:c>
       <x:c r="D25" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E25" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F25" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G25" t="str">
         <x:v>analyze</x:v>
       </x:c>
       <x:c r="H25" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I25" t="str">
         <x:v>python</x:v>
@@ -1703,50 +1664,53 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>algorithms</x:v>
+        <x:v>programming-fundamentals</x:v>
       </x:c>
       <x:c r="L25"/>
       <x:c r="M25" t="str">
-        <x:v>Only the second approach is a correct finite algorithm</x:v>
+        <x:v>Ask what “best” means before planning the solution</x:v>
       </x:c>
       <x:c r="N25" t="str">
-        <x:v>The first approach may never finish</x:v>
+        <x:v>Write the output screen before reading any records</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>The second approach can miss Ravi</x:v>
+        <x:v>Assume “best” always means the first record</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>Both are correct; the second is faster</x:v>
+        <x:v>Add every field together even though no weighting rule was supplied</x:v>
       </x:c>
       <x:c r="Q25" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
-        <x:v>Python - MCQ - 1.2.15</x:v>
+        <x:v>Python - MCQ - 1.3.5</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>A backup app wakes up on its own at 2 AM every night and runs, with no person typing anything at all.
-In the IPO model, what started it?</x:v>
+        <x:v>A customer-service procedure says:
+1. Ask whether the customer is satisfied.
+2. When the answer is no, say, “We will improve.”
+3. Return to step 1.
+Nothing changes, and there is no attempt limit. Which algorithm rule is not guaranteed?</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>Input is not only typing on a keyboard — it can be a tap, a file, a sensor reading, a network message, or a scheduled trigger. The 2 AM timer is a scheduled trigger, which is a form of input that set the program running.</x:v>
+        <x:v>Nothing guarantees that satisfaction will change or limits retries, so the procedure may never stop.</x:v>
       </x:c>
       <x:c r="D26" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E26" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F26" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H26" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I26" t="str">
         <x:v>python</x:v>
@@ -1755,20 +1719,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>inputs-processing-outputs</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L26"/>
       <x:c r="M26" t="str">
-        <x:v>Output</x:v>
+        <x:v>Effectiveness, because speaking is impossible</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>Processing</x:v>
+        <x:v>Input, because the customer gives an answer</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>No IPO stage</x:v>
+        <x:v>Output, because the procedure displays a message</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>Input</x:v>
+        <x:v>Finiteness, because the procedure has no guaranteed stopping point</x:v>
       </x:c>
       <x:c r="Q26" t="n">
         <x:v>4</x:v>
@@ -1776,17 +1740,16 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>Python - MCQ - 1.2.16</x:v>
+        <x:v>Python - MCQ - 1.3.6</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>On a flowchart, one shape is used for reading data in or showing a result out.
-Which shape is it?</x:v>
+        <x:v>A team writes one language-independent procedure for finding the largest of three numbers. Priya implements it in Python and Joel implements it in Java. Which statement correctly describes their work?</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>A parallelogram stands for input or output — reading data in or showing a result out. A diamond is a decision, an oval starts or ends the chart, and a rectangle is a plain process step.</x:v>
+        <x:v>The algorithm is the not tied to one programming language plan; each version written in a programming language is a program.</x:v>
       </x:c>
       <x:c r="D27" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E27" t="str">
         <x:v>published</x:v>
@@ -1795,10 +1758,10 @@
         <x:v>easy</x:v>
       </x:c>
       <x:c r="G27" t="str">
-        <x:v>remember</x:v>
+        <x:v>understand</x:v>
       </x:c>
       <x:c r="H27" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I27" t="str">
         <x:v>python</x:v>
@@ -1807,20 +1770,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K27" t="str">
-        <x:v>flowcharts</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L27"/>
       <x:c r="M27" t="str">
-        <x:v>Parallelogram</x:v>
+        <x:v>They use one algorithm but write two programs in different languages</x:v>
       </x:c>
       <x:c r="N27" t="str">
-        <x:v>Diamond</x:v>
+        <x:v>They have two unrelated algorithms because the syntax differs</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>Oval</x:v>
+        <x:v>The Python file is an algorithm, while the Java file is a program</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>Rectangle</x:v>
+        <x:v>Only compiled languages can express an algorithm</x:v>
       </x:c>
       <x:c r="Q27" t="n">
         <x:v>1</x:v>
@@ -1828,17 +1791,21 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
-        <x:v>Python - MCQ - 1.2.17</x:v>
+        <x:v>Python - MCQ - 1.3.7</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>A student cannot explain their plan for a task in plain language, yet keeps typing code and getting more confused.
-What does the problem-solving method say they should do?</x:v>
+        <x:v>A quality inspector checks `12`, `27`, and `19`:
+1. Store the first value.
+2. Compare the next value and keep the bigger one.
+3. Repeat for the last value.
+4. Report the stored value.
+What value is reported?</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>The rule is: understand first, plan second, build third. If you cannot explain your plan in plain language, the problem is not yet understood — the signal is to return to the Understand stage, not to type harder.</x:v>
+        <x:v>The stored largest changes from 12 to 27 and remains 27 because 19 is smaller.</x:v>
       </x:c>
       <x:c r="D28" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E28" t="str">
         <x:v>published</x:v>
@@ -1847,10 +1814,10 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G28" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H28" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I28" t="str">
         <x:v>python</x:v>
@@ -1859,20 +1826,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>problem-solving-approach</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L28"/>
       <x:c r="M28" t="str">
-        <x:v>Keep coding until a plan emerges</x:v>
+        <x:v>`12`, because the first value is stored first</x:v>
       </x:c>
       <x:c r="N28" t="str">
-        <x:v>Jump directly to final testing</x:v>
+        <x:v>`19`, because it is considered last</x:v>
       </x:c>
       <x:c r="O28" t="str">
-        <x:v>Return to understanding the problem</x:v>
+        <x:v>`27`, because it replaces `12` and is not replaced by `19`</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>Comment the existing code</x:v>
+        <x:v>`58`, because all measurements should be added</x:v>
       </x:c>
       <x:c r="Q28" t="n">
         <x:v>3</x:v>
@@ -1880,29 +1847,28 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
-        <x:v>Python - MCQ - 1.2.18</x:v>
+        <x:v>Python - MCQ - 1.3.8</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>A student needs to read data from the internet and does not want to build that ability from scratch. Python's design makes this easy.
-Which idea is this?</x:v>
+        <x:v>A phone has 20 contacts today but may have 20,000 next year. Method 1 checks each name from the top. Method 2 jumps to the correct letter before checking names. Both find the correct contact. Which statement is correct?</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>Python ships with a large set of ready-made tools ("batteries included"), and PyPI offers hundreds of thousands of free packages. So someone has usually built the hard part already, and you assemble the pieces instead of starting from zero.</x:v>
+        <x:v>Correctness and efficiency are separate. Both can find the contact, while the alphabetic index avoids many checks in a large list.</x:v>
       </x:c>
       <x:c r="D29" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E29" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F29" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G29" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H29" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I29" t="str">
         <x:v>python</x:v>
@@ -1911,20 +1877,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K29" t="str">
-        <x:v>why-python</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L29"/>
       <x:c r="M29" t="str">
-        <x:v>Indentation rules</x:v>
+        <x:v>Method 1 is the only algorithm because it checks every item</x:v>
       </x:c>
       <x:c r="N29" t="str">
-        <x:v>Mandatory compilation</x:v>
+        <x:v>Method 2 is incorrect because it skips unrelated letters</x:v>
       </x:c>
       <x:c r="O29" t="str">
-        <x:v>Small-program limitations</x:v>
+        <x:v>The methods must take the same time because both are correct</x:v>
       </x:c>
       <x:c r="P29" t="str">
-        <x:v>The standard library and PyPI</x:v>
+        <x:v>Both are correct, but Method 2 will probably be faster for a large list</x:v>
       </x:c>
       <x:c r="Q29" t="n">
         <x:v>4</x:v>
@@ -1932,17 +1898,16 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>Python - MCQ - 1.2.19</x:v>
+        <x:v>Python - MCQ - 1.3.9</x:v>
       </x:c>
       <x:c r="B30" t="str">
-        <x:v>Only one of the steps below is written clearly enough — with exactly one meaning — to belong in a real algorithm.
-Which step is it?</x:v>
+        <x:v>An ATM withdrawal procedure validates the PIN, checks the balance, dispenses cash, updates the balance, and ends. The requirement also states that the card must always be returned. Which problem must be fixed before release?</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>A real algorithm step must be definite: precise, with exactly one meaning. "Compare each pair of neighbours and swap them if they are out of order" can be read only one way. "Sort somehow", "make it nice", and "do the usual thing" are all too vague to act on.</x:v>
+        <x:v>Returning the card is an required step, so omitting it makes the instruction sequence incomplete.</x:v>
       </x:c>
       <x:c r="D30" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E30" t="str">
         <x:v>published</x:v>
@@ -1954,7 +1919,7 @@
         <x:v>analyze</x:v>
       </x:c>
       <x:c r="H30" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I30" t="str">
         <x:v>python</x:v>
@@ -1963,20 +1928,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K30" t="str">
-        <x:v>algorithms</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L30"/>
       <x:c r="M30" t="str">
-        <x:v>Compare neighbouring items and swap misplaced pairs</x:v>
+        <x:v>The procedure is missing the required step that returns the card</x:v>
       </x:c>
       <x:c r="N30" t="str">
-        <x:v>Arrange the values into a suitable order somehow</x:v>
+        <x:v>The procedure is ambiguous because “cash” has no meaning</x:v>
       </x:c>
       <x:c r="O30" t="str">
-        <x:v>Improve the list until its order looks acceptable</x:v>
+        <x:v>The procedure is infinite because it updates the balance</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>Use the usual method for organising the numbers</x:v>
+        <x:v>The procedure has no processing because it uses a PIN</x:v>
       </x:c>
       <x:c r="Q30" t="n">
         <x:v>1</x:v>
@@ -1984,17 +1949,22 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
-        <x:v>Python - MCQ - 1.2.20</x:v>
+        <x:v>Python - MCQ - 1.3.10</x:v>
       </x:c>
       <x:c r="B31" t="str">
-        <x:v>In pseudocode, the keywords BEGIN and END are used at the top and bottom of the logic.
-What is their job?</x:v>
+        <x:v>A team writes this during a design meeting:
+```text
+READ marks
+COMPUTE average
+PRINT average
+```
+The plan is clear to the team, but the computer cannot run it directly. What is this plan?</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>BEGIN and END are boundary keywords: they mark where the logic starts and stops. READ and PRINT handle input and output, FOR and WHILE handle repetition, and IF handles a decision.</x:v>
+        <x:v>It is pseudocode. It shows the planned steps for people to review before they write real code.</x:v>
       </x:c>
       <x:c r="D31" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E31" t="str">
         <x:v>published</x:v>
@@ -2003,10 +1973,10 @@
         <x:v>easy</x:v>
       </x:c>
       <x:c r="G31" t="str">
-        <x:v>remember</x:v>
+        <x:v>understand</x:v>
       </x:c>
       <x:c r="H31" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 3</x:v>
       </x:c>
       <x:c r="I31" t="str">
         <x:v>python</x:v>
@@ -2015,20 +1985,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K31" t="str">
-        <x:v>pseudocode</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L31"/>
       <x:c r="M31" t="str">
-        <x:v>Handling input and output</x:v>
+        <x:v>A finished Python program</x:v>
       </x:c>
       <x:c r="N31" t="str">
-        <x:v>Marking the logic's boundaries</x:v>
+        <x:v>Pseudocode that people can review before writing code</x:v>
       </x:c>
       <x:c r="O31" t="str">
-        <x:v>Repeating a block</x:v>
+        <x:v>A flowchart without shapes</x:v>
       </x:c>
       <x:c r="P31" t="str">
-        <x:v>Selecting between alternatives</x:v>
+        <x:v>A saved program with the wrong file name</x:v>
       </x:c>
       <x:c r="Q31" t="n">
         <x:v>2</x:v>
@@ -2036,17 +2006,16 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
-        <x:v>Python - MCQ - 1.2.21</x:v>
+        <x:v>Python - MCQ - 1.4.1</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>A tea recipe lists the steps as: (1) pour into a cup, (2) boil the water, (3) add the tea powder. Followed exactly, it gives a poor result.
-What is wrong with these instructions?</x:v>
+        <x:v>A draft solution tries to calculate `average` before receiving any marks. Which pseudocode uses the correct order?</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>Good instructions must be ordered — the sequence matters. Here the steps are simply in the wrong order: you cannot pour the tea into a cup before the water is even boiled. No step is missing or ambiguous; they are just out of sequence.</x:v>
+        <x:v>The marks must be received before the average can be computed and shown.</x:v>
       </x:c>
       <x:c r="D32" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E32" t="str">
         <x:v>published</x:v>
@@ -2055,10 +2024,10 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G32" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H32" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I32" t="str">
         <x:v>python</x:v>
@@ -2067,50 +2036,80 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K32" t="str">
-        <x:v>what-is-programming</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L32"/>
       <x:c r="M32" t="str">
-        <x:v>The actions are in the wrong sequence</x:v>
+        <x:v>```text
+BEGIN
+    PRINT average
+    READ mark1, mark2, mark3
+END
+```</x:v>
       </x:c>
       <x:c r="N32" t="str">
-        <x:v>A required action is omitted</x:v>
+        <x:v>```text
+BEGIN
+    SET average = (mark1 + mark2 + mark3) / 3
+    READ mark1, mark2, mark3
+    PRINT average
+END
+```</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>One action has two possible interpretations</x:v>
+        <x:v>```text
+BEGIN
+    READ mark1, mark2, mark3
+    SET average = (mark1 + mark2 + mark3) / 3
+    PRINT average
+END
+```</x:v>
       </x:c>
       <x:c r="P32" t="str">
-        <x:v>Unnecessary actions are included</x:v>
+        <x:v>```text
+BEGIN
+    READ average
+    PRINT mark1, mark2, mark3
+END
+```</x:v>
       </x:c>
       <x:c r="Q32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>Python - MCQ - 1.2.22</x:v>
+        <x:v>Python - MCQ - 1.4.2</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>You just want a quick, throwaway answer to "what is 1234 times 5678?" right now, with nothing to save.
-Which tool fits best?</x:v>
+        <x:v>A delivery team reviews this pseudocode:
+```text
+BEGIN
+    READ order_total
+    SET delivery_fee = 50
+    SET final_total = order_total + delivery_fee
+    PRINT final_total
+END
+```
+The order total is ₹500. What should the review record show?</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>The REPL (Python's interactive shell) is made for quick, throwaway questions — you type the calculation and the answer appears at once, with nothing to save. A script is better when you want to keep and rerun something.</x:v>
+        <x:v>The plan adds the ₹50 delivery fee to ₹500 and displays ₹550.</x:v>
       </x:c>
       <x:c r="D33" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E33" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F33" t="str">
-        <x:v>easy</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G33" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H33" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I33" t="str">
         <x:v>python</x:v>
@@ -2119,38 +2118,37 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K33" t="str">
-        <x:v>setting-up-python-first-program</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L33"/>
       <x:c r="M33" t="str">
-        <x:v>The interactive REPL</x:v>
+        <x:v>₹50 is displayed</x:v>
       </x:c>
       <x:c r="N33" t="str">
-        <x:v>A reusable saved script</x:v>
+        <x:v>₹500 is displayed</x:v>
       </x:c>
       <x:c r="O33" t="str">
-        <x:v>A calculation flowchart</x:v>
+        <x:v>Nothing is displayed</x:v>
       </x:c>
       <x:c r="P33" t="str">
-        <x:v>Calculation pseudocode</x:v>
+        <x:v>₹550 is displayed</x:v>
       </x:c>
       <x:c r="Q33" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>Python - MCQ - 1.2.23</x:v>
+        <x:v>Python - MCQ - 1.4.3</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>After breaking a problem down, spotting its repeating pattern, and ignoring the noise, one last step turns it into a precise, ordered sequence of steps.
-What is that step called?</x:v>
+        <x:v>A login design should show “Welcome” for a correct PIN and “Try again” for an incorrect PIN. Which plain-language plan shows the two results clearly?</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>Turning your decomposed, pattern-spotted, abstracted problem into a precise, ordered sequence of steps is algorithmic thinking — often named as the fourth pillar. It leads directly to writing an actual algorithm.</x:v>
+        <x:v>The correct plan connects each PIN result to the correct message.</x:v>
       </x:c>
       <x:c r="D34" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E34" t="str">
         <x:v>published</x:v>
@@ -2159,10 +2157,10 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G34" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H34" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I34" t="str">
         <x:v>python</x:v>
@@ -2171,50 +2169,49 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K34" t="str">
-        <x:v>computational-thinking</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L34"/>
       <x:c r="M34" t="str">
-        <x:v>Removing details that do not matter</x:v>
+        <x:v>Show both messages for every PIN</x:v>
       </x:c>
       <x:c r="N34" t="str">
-        <x:v>Splitting the task into smaller parts</x:v>
+        <x:v>Show Try again first, then always show Welcome</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>Recognising repeated problem shapes</x:v>
+        <x:v>Correct PIN: show Welcome; incorrect PIN: show Try again</x:v>
       </x:c>
       <x:c r="P34" t="str">
-        <x:v>Turning the solution into ordered steps</x:v>
+        <x:v>Correct PIN: show Try again; incorrect PIN: show Welcome</x:v>
       </x:c>
       <x:c r="Q34" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>Python - MCQ - 1.2.24</x:v>
+        <x:v>Python - MCQ - 1.4.4</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>Compared with a typical compiled language such as C or Java, how does Python usually get from written code to running?
-Which statement is correct?</x:v>
+        <x:v>A chart must read marks, calculate an average, decide whether the average is at least 40, and display Pass or Fail. Which set of flowchart shapes is correct?</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>Python runs your code almost immediately, without a separate compile step first. A typical compiled language is usually turned into machine code in a separate step before it can run.</x:v>
+        <x:v>Parallelograms represent input/output, rectangles represent processing, and diamonds represent decisions.</x:v>
       </x:c>
       <x:c r="D35" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E35" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F35" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G35" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H35" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I35" t="str">
         <x:v>python</x:v>
@@ -2223,38 +2220,37 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K35" t="str">
-        <x:v>why-python</x:v>
+        <x:v>flowcharts</x:v>
       </x:c>
       <x:c r="L35"/>
       <x:c r="M35" t="str">
-        <x:v>It always requires a separate compilation step</x:v>
+        <x:v>Read marks: parallelogram; calculate average: rectangle; threshold question: diamond; display result: parallelogram</x:v>
       </x:c>
       <x:c r="N35" t="str">
-        <x:v>It must first be rewritten in another language</x:v>
+        <x:v>Read marks: diamond; calculate average: oval; threshold question: rectangle; display result: arrow</x:v>
       </x:c>
       <x:c r="O35" t="str">
-        <x:v>It runs without a separate compile command</x:v>
+        <x:v>Read marks: rectangle; calculate average: parallelogram; threshold question: oval; display result: diamond</x:v>
       </x:c>
       <x:c r="P35" t="str">
-        <x:v>It runs only through a web browser</x:v>
+        <x:v>Use rectangles for every step because the arrows already show direction</x:v>
       </x:c>
       <x:c r="Q35" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
-        <x:v>Python - MCQ - 1.2.25</x:v>
+        <x:v>Python - MCQ - 1.4.5</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>A beginner writes `print(Welcome)` without quotation marks around the word, and gets an error.
-Why?</x:v>
+        <x:v>A railway turnstile flowchart has a diamond labelled `Ticket valid?`. Its two outgoing arrows are not labelled, so a reader cannot tell which path opens the gate. How should the chart be made clear?</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>Text you want to show must be wrapped in quotes. Without them, Python treats `Welcome` as a name or command to look up rather than as a message to display, so it errors. Writing `print("Welcome")` fixes it.</x:v>
+        <x:v>A decision needs labelled outcomes so readers can connect each result to the correct next action.</x:v>
       </x:c>
       <x:c r="D36" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E36" t="str">
         <x:v>published</x:v>
@@ -2266,7 +2262,7 @@
         <x:v>analyze</x:v>
       </x:c>
       <x:c r="H36" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I36" t="str">
         <x:v>python</x:v>
@@ -2275,20 +2271,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K36" t="str">
-        <x:v>setting-up-python-first-program</x:v>
+        <x:v>flowcharts</x:v>
       </x:c>
       <x:c r="L36"/>
       <x:c r="M36" t="str">
-        <x:v>print accepts numeric values but not text</x:v>
+        <x:v>Remove one outgoing arrow</x:v>
       </x:c>
       <x:c r="N36" t="str">
-        <x:v>Welcome is treated as a variable name</x:v>
+        <x:v>Label the outgoing paths `Yes` and `No` and connect each to its corresponding action</x:v>
       </x:c>
       <x:c r="O36" t="str">
-        <x:v>print cannot display a single word</x:v>
+        <x:v>Replace the diamond with a process rectangle</x:v>
       </x:c>
       <x:c r="P36" t="str">
-        <x:v>The statement needs a semicolon</x:v>
+        <x:v>Put both outcomes on one arrow</x:v>
       </x:c>
       <x:c r="Q36" t="n">
         <x:v>2</x:v>
@@ -2296,29 +2292,28 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
-        <x:v>Python - MCQ - 1.2.26</x:v>
+        <x:v>Python - MCQ - 1.4.6</x:v>
       </x:c>
       <x:c r="B37" t="str">
-        <x:v>A program prints 5,000 fee receipts in under a second, every one correct, while a tired clerk would take days by hand and make mistakes.
-What did the programmer do that the clerk did not?</x:v>
+        <x:v>A login flowchart allows three password attempts. After a wrong password, it returns for another attempt while attempts remain. A user enters two wrong passwords and then the correct password. What path does the user follow?</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>The programmer stopped doing the work and started describing it: capturing the task as a clear, ordered set of instructions the computer can carry out again and again. The computer supplies the speed; the programmer supplies the thinking — no advanced maths required.</x:v>
+        <x:v>The chart returns after the first two failures. The correct third password follows the success path with two failed attempts recorded.</x:v>
       </x:c>
       <x:c r="D37" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E37" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F37" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G37" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H37" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I37" t="str">
         <x:v>python</x:v>
@@ -2327,50 +2322,49 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K37" t="str">
-        <x:v>what-is-programming</x:v>
+        <x:v>flowcharts</x:v>
       </x:c>
       <x:c r="L37"/>
       <x:c r="M37" t="str">
-        <x:v>Completed the manual work more quickly</x:v>
+        <x:v>The account locks after the second failure because only two retries are allowed</x:v>
       </x:c>
       <x:c r="N37" t="str">
-        <x:v>Removed all need for human reasoning</x:v>
+        <x:v>The success is ignored because any earlier failure forces the lock path</x:v>
       </x:c>
       <x:c r="O37" t="str">
-        <x:v>Defined repeatable instructions once</x:v>
+        <x:v>The chart never stops because every backward arrow is infinite</x:v>
       </x:c>
       <x:c r="P37" t="str">
-        <x:v>Applied advanced mathematics to each receipt</x:v>
+        <x:v>It returns after each of the first two failures, then follows the success path</x:v>
       </x:c>
       <x:c r="Q37" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
-        <x:v>Python - MCQ - 1.2.27</x:v>
+        <x:v>Python - MCQ - 1.4.7</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>You are designing a shopping-bill total. Your plan: ask for the price and quantity, multiply them together, then show the total.
-Which part is the processing step?</x:v>
+        <x:v>A developer needs to plan a short salary calculation, edit its steps quickly, and discuss it with another developer. It has one simple sequence and no complicated web of branches. Which tool is best for this task?</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>Asking for the price and quantity is input, and showing the total is output. Multiplying price by quantity is the calculation in the middle — the processing step. The same processing works for any values the user enters.</x:v>
+        <x:v>Pseudocode is quick to draft and edit when the purpose is to reason about mostly sequential logic before implementation.</x:v>
       </x:c>
       <x:c r="D38" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E38" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F38" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G38" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H38" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I38" t="str">
         <x:v>python</x:v>
@@ -2379,20 +2373,20 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K38" t="str">
-        <x:v>inputs-processing-outputs</x:v>
+        <x:v>algorithms-and-pseudocode</x:v>
       </x:c>
       <x:c r="L38"/>
       <x:c r="M38" t="str">
-        <x:v>Collecting the price and quantity</x:v>
+        <x:v>Build the full graphical interface first</x:v>
       </x:c>
       <x:c r="N38" t="str">
-        <x:v>Displaying the calculated total</x:v>
+        <x:v>Draw a large flowchart even though the path never branches</x:v>
       </x:c>
       <x:c r="O38" t="str">
-        <x:v>Calculating price multiplied by quantity</x:v>
+        <x:v>Write concise pseudocode, then trace and translate it later</x:v>
       </x:c>
       <x:c r="P38" t="str">
-        <x:v>Storing the completed bill permanently</x:v>
+        <x:v>Avoid planning because sequential problems cannot contain mistakes</x:v>
       </x:c>
       <x:c r="Q38" t="n">
         <x:v>3</x:v>
@@ -2400,17 +2394,16 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
-        <x:v>Python - MCQ - 1.2.28</x:v>
+        <x:v>Python - MCQ - 1.4.8</x:v>
       </x:c>
       <x:c r="B39" t="str">
-        <x:v>Trace this algorithm for the numbers 12, 27, and 19: assume the first number is the largest; if the second is bigger, it becomes the largest; if the third is bigger, it becomes the largest.
-What is the final answer, and why is it guaranteed to finish?</x:v>
+        <x:v>A team is building a small device controller with extremely limited memory and very strict timing needs. Another team is building a data-analysis trial project. Which choice best fits the two projects?</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>Start with 12. Is 27 bigger? Yes, so the largest becomes 27. Is 19 bigger than 27? No, so it stays 27. The answer is 27. It always finishes because it makes a fixed number of comparisons, no matter what the numbers are — that is its finiteness.</x:v>
+        <x:v>Python fits rapid data work, while small systems with strict memory and timing limits may benefit from a lower-level compiled language.</x:v>
       </x:c>
       <x:c r="D39" t="n">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E39" t="str">
         <x:v>published</x:v>
@@ -2419,10 +2412,10 @@
         <x:v>hard</x:v>
       </x:c>
       <x:c r="G39" t="str">
-        <x:v>apply</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H39" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I39" t="str">
         <x:v>python</x:v>
@@ -2431,38 +2424,42 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K39" t="str">
-        <x:v>algorithms</x:v>
+        <x:v>python-overview</x:v>
       </x:c>
       <x:c r="L39"/>
       <x:c r="M39" t="str">
-        <x:v>19; the final number always replaces earlier ones</x:v>
+        <x:v>Python must be selected for both because readable languages are always fastest</x:v>
       </x:c>
       <x:c r="N39" t="str">
-        <x:v>27; only two comparisons are required</x:v>
+        <x:v>A compiled language must be selected for both because Python has no real-world uses</x:v>
       </x:c>
       <x:c r="O39" t="str">
-        <x:v>12; the initial number can never change</x:v>
+        <x:v>Language choice never depends on the task</x:v>
       </x:c>
       <x:c r="P39" t="str">
-        <x:v>No result; the comparisons repeat indefinitely</x:v>
+        <x:v>Python suits the data project, while a lower-level language may suit the small controller better</x:v>
       </x:c>
       <x:c r="Q39" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="str">
-        <x:v>Python - MCQ - 1.2.29</x:v>
+        <x:v>Python - MCQ - 1.4.9</x:v>
       </x:c>
       <x:c r="B40" t="str">
-        <x:v>A flowchart has a decision diamond "Average 40 or more?" but only one arrow leaves it, and that arrow has no label.
-What is the problem?</x:v>
+        <x:v>A beginner runs this saved script:
+```python
+print("Welcome")
+score = 10 + 5
+```
+The learner expected to see both `Welcome` and `15`. Which explanation is correct?</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>Every decision diamond must have a labelled exit for each outcome (such as yes and no). With one unlabelled arrow, the reader is left guessing what happens for each answer. The diamond itself is the right shape for a decision.</x:v>
+        <x:v>The assignment calculates and stores the value, but only `print` sends a value to the screen in a script.</x:v>
       </x:c>
       <x:c r="D40" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E40" t="str">
         <x:v>published</x:v>
@@ -2474,7 +2471,7 @@
         <x:v>analyze</x:v>
       </x:c>
       <x:c r="H40" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I40" t="str">
         <x:v>python</x:v>
@@ -2483,50 +2480,54 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K40" t="str">
-        <x:v>flowcharts</x:v>
+        <x:v>python-environment</x:v>
       </x:c>
       <x:c r="L40"/>
       <x:c r="M40" t="str">
-        <x:v>Diamonds cannot contain questions</x:v>
+        <x:v>The calculation never occurs because assignment is not processing</x:v>
       </x:c>
       <x:c r="N40" t="str">
-        <x:v>Every decision needs at least three exits</x:v>
+        <x:v>`Welcome` appears, and `15` is stored but not displayed because no `print` instruction outputs `score`</x:v>
       </x:c>
       <x:c r="O40" t="str">
-        <x:v>The outcomes are missing distinct branch labels</x:v>
+        <x:v>Python automatically displays every stored value in a script</x:v>
       </x:c>
       <x:c r="P40" t="str">
-        <x:v>Flowcharts cannot contain decisions</x:v>
+        <x:v>The script must be moved into the REPL before assignment can work</x:v>
       </x:c>
       <x:c r="Q40" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="str">
-        <x:v>Python - MCQ - 1.2.30</x:v>
+        <x:v>Python - MCQ - 1.4.10</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>A capable student avoids programming, believing "you must be a maths genius, and you must memorise everything".
-Based on this unit, what is the honest response?</x:v>
+        <x:v>A welcome kiosk contains:
+```python
+age = input("Age: ")
+print(age + age)
+```
+A visitor types `20`. The designer expected `40`, but the screen shows `2020`. Which change is correct?</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>Neither belief is true. For most programming, school arithmetic is plenty — the real skill is logical, step-by-step thinking. And you do not memorise everything: even professionals look things up constantly. Programming is a skill built through practice.</x:v>
+        <x:v>`input()` returns a string, so `+` joins `"20"` and `"20"`; the input must first be converted to a number for addition.</x:v>
       </x:c>
       <x:c r="D41" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E41" t="str">
         <x:v>published</x:v>
       </x:c>
       <x:c r="F41" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G41" t="str">
-        <x:v>understand</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H41" t="str">
-        <x:v>python - Set 2</x:v>
+        <x:v>python - Set 4</x:v>
       </x:c>
       <x:c r="I41" t="str">
         <x:v>python</x:v>
@@ -2535,23 +2536,24 @@
         <x:v>introduction-to-programming</x:v>
       </x:c>
       <x:c r="K41" t="str">
-        <x:v>what-is-programming</x:v>
+        <x:v>python-environment</x:v>
       </x:c>
       <x:c r="L41"/>
       <x:c r="M41" t="str">
-        <x:v>Both beliefs are correct</x:v>
+        <x:v>Replace `print` because it turns every number into repeated text</x:v>
       </x:c>
       <x:c r="N41" t="str">
-        <x:v>Neither belief is required</x:v>
+        <x:v>Run the same file from the REPL because scripts cannot add numbers</x:v>
       </x:c>
       <x:c r="O41" t="str">
-        <x:v>Only memorisation is required</x:v>
+        <x:v>Recognise that `input` supplied the text `"20"`; convert it to a numeric value before performing addition</x:v>
       </x:c>
       <x:c r="P41" t="str">
-        <x:v>Only exceptional mathematics is required</x:v>
+        <x:v>Save the input in storage before using it so RAM can calculate correctly
+---</x:v>
       </x:c>
       <x:c r="Q41" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>